<commit_message>
update CR week 18 y varios
</commit_message>
<xml_diff>
--- a/checkrates/week-18/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-18/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6161,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -8004,7 +8004,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10185,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -12123,7 +12123,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -12276,7 +12276,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -12429,7 +12429,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -12588,7 +12588,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -14686,7 +14686,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -16629,7 +16629,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -18572,7 +18572,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -20415,7 +20415,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -22258,7 +22258,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -22701,7 +22701,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -24639,7 +24639,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -24798,7 +24798,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -26891,7 +26891,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -27050,7 +27050,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -29148,7 +29148,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -31091,7 +31091,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -33034,7 +33034,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -34877,7 +34877,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -36720,7 +36720,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -37196,7 +37196,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -39139,7 +39139,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -41081,7 +41081,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -42869,7 +42869,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -44712,7 +44712,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -46555,7 +46555,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -47031,7 +47031,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:12 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>